<commit_message>
Add 2 terms to BCIO_Upper_Rels.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Rels.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Rels.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1426,22 +1426,23 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BFO:0000054</t>
+          <t>AFO:0000062</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>realised in</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>realized in [BFO:0000054]</t>
+          <t>preceded by</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>temporally related to [RO:0002222]</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Inverse of realizes relation.</t>
+          <t>x is preceded by y if and only if the time point at which y ends is before or equivalent to the time point at which x starts. Formally: x preceded by y iff ω(y) &lt;= α(x), where α is a function that maps a process to a start point, and ω is a function that maps a process to an end point.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1454,83 +1455,150 @@
           <t>occurrent</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BFO:0000055</t>
+          <t>AFO:0000063</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>realises</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>realizes [BFO:0000055]</t>
+          <t>precedes</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>temporally related to [RO:0002222]</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>To say that b realizes c at t is to assert that there is some material entity d and b is a process which has participant d at t and c is a disposition or role of which d is bearer_of at tand the type instantiated by b is correlated with the type instantiated by c.</t>
-        </is>
-      </c>
+          <t>x precedes y if and only if the time point at which x ends is before or equivalent to the time point at which y starts. Formally: x precedes y iff ω(x) &lt;= α(y), where α is a function that maps a process to a start point, and ω is a function that maps a process to an end point.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>occurrent</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BCIOR:000008</t>
+          <t>BFO:0000054</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>through</t>
+          <t>realised in</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>realized in [BFO:0000054]</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>A relation that holds between an behaviour change intervention mechanism of action and an entity (x), if (1) x participates in or is part of the mechanism of action process and (2) x is influenced by the behavior change intervention in some scenario such that there is some change in entity x.</t>
+          <t>Inverse of realizes relation.</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>behaviour change intervention mechanism of action</t>
+          <t>occurrent</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>entity [BFO:0000001]</t>
+          <t>occurrent</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>BFO:0000055</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>realises</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>realizes [BFO:0000055]</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>To say that b realizes c at t is to assert that there is some material entity d and b is a process which has participant d at t and c is a disposition or role of which d is bearer_of at tand the type instantiated by b is correlated with the type instantiated by c.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BCIOR:000008</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>through</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>A relation that holds between an behaviour change intervention mechanism of action and an entity (x), if (1) x participates in or is part of the mechanism of action process and (2) x is influenced by the behavior change intervention in some scenario such that there is some change in entity x.</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>behaviour change intervention mechanism of action</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>entity [BFO:0000001]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>BCIOR:000015</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>uses</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>has participant [RO:0000057]</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Has participant that relates a behaviour to a material entity that the person enacting the behaviour intends to enable or facilitate the behaviour.</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>individual human behaviour</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>material entity</t>
         </is>

</xml_diff>

<commit_message>
Update 2 terms in BCIO_Upper_Rels.xlsx
</commit_message>
<xml_diff>
--- a/Upper Level BCIO/inputs/BCIO_Upper_Rels.xlsx
+++ b/Upper Level BCIO/inputs/BCIO_Upper_Rels.xlsx
@@ -1426,7 +1426,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AFO:0000062</t>
+          <t>BFO:0000062</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1434,7 +1434,6 @@
           <t>preceded by</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr"/>
       <c r="D37" t="inlineStr">
         <is>
           <t>temporally related to [RO:0002222]</t>
@@ -1455,12 +1454,11 @@
           <t>occurrent</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AFO:0000063</t>
+          <t>BFO:0000063</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1468,7 +1466,6 @@
           <t>precedes</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
           <t>temporally related to [RO:0002222]</t>
@@ -1489,7 +1486,6 @@
           <t>occurrent</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">

</xml_diff>